<commit_message>
DO and EFO update
</commit_message>
<xml_diff>
--- a/data-raw/metadata_phen_oncox.xlsx
+++ b/data-raw/metadata_phen_oncox.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__phenOncoX/phenOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C0CAC6-4341-E349-B9FE-40E1049B156E}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193D17F6-7771-F948-A2B4-50CFFB71FD3B}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="920" yWindow="3320" windowWidth="34920" windowHeight="19080" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
@@ -153,10 +153,10 @@
     <t>2025_10_03</t>
   </si>
   <si>
-    <t>v2026-08-31</t>
-  </si>
-  <si>
-    <t>v3.94.0</t>
+    <t>v3.95.0</t>
+  </si>
+  <si>
+    <t>v2026-09-30</t>
   </si>
 </sst>
 </file>
@@ -639,7 +639,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -665,7 +665,7 @@
         <v>14</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>

</xml_diff>